<commit_message>
Deploy 2026-07-03 QA sessions: map layers UI, autoscroll, and click fixes.
Adds MapLayerPanel for map navigation, unified bottom Слои panel with nested category toggles, element-level autoscroll with layer switch throttle, mount/activity click overrides, mobile legend positioning, and splash modal polish.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/new_legend/longread (2).xlsx
+++ b/new_legend/longread (2).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\SPb_Mountains\SPb_Mountains\new_legend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2E8325-2CAA-40D4-AF5D-A3CE4FC7D2E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69A72136-2093-4129-84B4-FF32D91CCF4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LONGREAD" sheetId="1" r:id="rId1"/>
@@ -1988,21 +1988,21 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:N1006"/>
-  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="22.73046875" customWidth="1"/>
-    <col min="2" max="2" width="20.46484375" customWidth="1"/>
-    <col min="3" max="3" width="16.86328125" customWidth="1"/>
-    <col min="4" max="4" width="8.59765625" customWidth="1"/>
-    <col min="5" max="5" width="50.3984375" customWidth="1"/>
-    <col min="6" max="6" width="20.86328125" customWidth="1"/>
-    <col min="7" max="7" width="16.46484375" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" customWidth="1"/>
+    <col min="5" max="5" width="50.42578125" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" customWidth="1"/>
     <col min="8" max="8" width="21" customWidth="1"/>
-    <col min="9" max="9" width="24.1328125" customWidth="1"/>
-    <col min="10" max="10" width="29.1328125" customWidth="1"/>
-    <col min="11" max="11" width="14.265625" customWidth="1"/>
+    <col min="9" max="9" width="24.140625" customWidth="1"/>
+    <col min="10" max="10" width="29.140625" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="61.3984375" customWidth="1"/>
+    <col min="13" max="13" width="61.42578125" customWidth="1"/>
     <col min="14" max="29" width="11" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2050,7 +2050,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="39.4">
+    <row r="2" spans="1:14" ht="38.25">
       <c r="A2" s="5" t="s">
         <v>14</v>
       </c>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="N2" s="12"/>
     </row>
-    <row r="3" spans="1:14" ht="64.5">
+    <row r="3" spans="1:14" ht="76.5">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="7">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="N3" s="12"/>
     </row>
-    <row r="4" spans="1:14" ht="39">
+    <row r="4" spans="1:14" ht="38.25">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="7">
@@ -2153,7 +2153,7 @@
       <c r="M5" s="7"/>
       <c r="N5" s="12"/>
     </row>
-    <row r="6" spans="1:14" ht="64.5">
+    <row r="6" spans="1:14" ht="63.75">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="7">
@@ -2223,7 +2223,7 @@
       <c r="M8" s="7"/>
       <c r="N8" s="12"/>
     </row>
-    <row r="9" spans="1:14" ht="25.9">
+    <row r="9" spans="1:14" ht="25.5">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="7">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N12" s="12"/>
     </row>
-    <row r="13" spans="1:14" ht="64.900000000000006">
+    <row r="13" spans="1:14" ht="63.75">
       <c r="A13" s="6"/>
       <c r="B13" s="5"/>
       <c r="C13" s="7">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="N17" s="12"/>
     </row>
-    <row r="18" spans="1:14" ht="38.25">
+    <row r="18" spans="1:14" ht="51">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="8">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="N20" s="12"/>
     </row>
-    <row r="21" spans="1:14" ht="90">
+    <row r="21" spans="1:14" ht="89.25">
       <c r="A21" s="6" t="s">
         <v>51</v>
       </c>
@@ -2583,7 +2583,7 @@
       <c r="M23" s="7"/>
       <c r="N23" s="12"/>
     </row>
-    <row r="24" spans="1:14" ht="26.25">
+    <row r="24" spans="1:14" ht="25.5">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="8">
@@ -2648,7 +2648,7 @@
       <c r="L26" s="14"/>
       <c r="M26" s="14"/>
     </row>
-    <row r="27" spans="1:14" ht="13.15">
+    <row r="27" spans="1:14" ht="25.5">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="8">
@@ -2670,7 +2670,7 @@
       <c r="M27" s="10"/>
       <c r="N27" s="12"/>
     </row>
-    <row r="28" spans="1:14" ht="51.4">
+    <row r="28" spans="1:14" ht="51">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7">
@@ -2735,7 +2735,7 @@
       <c r="M30" s="7"/>
       <c r="N30" s="12"/>
     </row>
-    <row r="31" spans="1:14" ht="26.25">
+    <row r="31" spans="1:14" ht="25.5">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="7"/>
@@ -2755,7 +2755,7 @@
       <c r="M31" s="7"/>
       <c r="N31" s="12"/>
     </row>
-    <row r="32" spans="1:14" ht="38.65">
+    <row r="32" spans="1:14" ht="51">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="7">
@@ -2803,7 +2803,7 @@
       <c r="M33" s="7"/>
       <c r="N33" s="12"/>
     </row>
-    <row r="34" spans="1:14" ht="26.25">
+    <row r="34" spans="1:14" ht="25.5">
       <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="7"/>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="N36" s="12"/>
     </row>
-    <row r="37" spans="1:14" ht="105">
+    <row r="37" spans="1:14" ht="127.5">
       <c r="A37" s="6" t="s">
         <v>75</v>
       </c>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="N37" s="12"/>
     </row>
-    <row r="38" spans="1:14" ht="64.150000000000006">
+    <row r="38" spans="1:14" ht="76.5">
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="7">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="N38" s="12"/>
     </row>
-    <row r="39" spans="1:14" ht="90.4">
+    <row r="39" spans="1:14" ht="89.25">
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="7">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="N39" s="12"/>
     </row>
-    <row r="40" spans="1:14" ht="38.65">
+    <row r="40" spans="1:14" ht="38.25">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="7">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="N40" s="12"/>
     </row>
-    <row r="41" spans="1:14" ht="63.75">
+    <row r="41" spans="1:14" ht="76.5">
       <c r="A41" s="6"/>
       <c r="B41" s="6" t="s">
         <v>82</v>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="N41" s="12"/>
     </row>
-    <row r="42" spans="1:14" ht="103.15">
+    <row r="42" spans="1:14" ht="102">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="7">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="N42" s="12"/>
     </row>
-    <row r="43" spans="1:14" ht="89.65">
+    <row r="43" spans="1:14" ht="89.25">
       <c r="A43" s="6"/>
       <c r="B43" s="6" t="s">
         <v>88</v>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="N44" s="12"/>
     </row>
-    <row r="45" spans="1:14" ht="128.25">
+    <row r="45" spans="1:14" ht="140.25">
       <c r="A45" s="6" t="s">
         <v>97</v>
       </c>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="N46" s="12"/>
     </row>
-    <row r="47" spans="1:14" ht="102">
+    <row r="47" spans="1:14" ht="114.75">
       <c r="A47" s="6"/>
       <c r="B47" s="6"/>
       <c r="C47" s="7">
@@ -3187,7 +3187,7 @@
       <c r="M47" s="7"/>
       <c r="N47" s="12"/>
     </row>
-    <row r="48" spans="1:14" ht="115.9">
+    <row r="48" spans="1:14" ht="114.75">
       <c r="A48" s="6"/>
       <c r="B48" s="6" t="s">
         <v>108</v>
@@ -3273,7 +3273,7 @@
       <c r="M50" s="7"/>
       <c r="N50" s="12"/>
     </row>
-    <row r="51" spans="1:14" ht="102.75">
+    <row r="51" spans="1:14" ht="114.75">
       <c r="A51" s="6"/>
       <c r="B51" s="6"/>
       <c r="C51" s="7">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="N51" s="12"/>
     </row>
-    <row r="52" spans="1:14" ht="76.5">
+    <row r="52" spans="1:14" ht="89.25">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="7">
@@ -3371,7 +3371,7 @@
       </c>
       <c r="N53" s="12"/>
     </row>
-    <row r="54" spans="1:14" ht="115.5">
+    <row r="54" spans="1:14" ht="114.75">
       <c r="A54" s="6"/>
       <c r="B54" s="5" t="s">
         <v>126</v>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="N54" s="12"/>
     </row>
-    <row r="55" spans="1:14" ht="77.25">
+    <row r="55" spans="1:14" ht="89.25">
       <c r="A55" s="6"/>
       <c r="B55" s="5"/>
       <c r="C55" s="7">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="N55" s="12"/>
     </row>
-    <row r="56" spans="1:14" ht="51">
+    <row r="56" spans="1:14" ht="63.75">
       <c r="A56" s="6" t="s">
         <v>130</v>
       </c>
@@ -3459,7 +3459,7 @@
       </c>
       <c r="N56" s="12"/>
     </row>
-    <row r="57" spans="1:14" ht="64.5">
+    <row r="57" spans="1:14" ht="76.5">
       <c r="A57" s="6"/>
       <c r="B57" s="5"/>
       <c r="C57" s="7">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="N57" s="12"/>
     </row>
-    <row r="58" spans="1:14" ht="103.9">
+    <row r="58" spans="1:14" ht="117.75">
       <c r="A58" s="6"/>
       <c r="B58" s="5"/>
       <c r="C58" s="7">
@@ -17750,16 +17750,16 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Z1074"/>
-  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.265625" customWidth="1"/>
-    <col min="2" max="2" width="27.265625" customWidth="1"/>
-    <col min="3" max="3" width="27.59765625" customWidth="1"/>
-    <col min="4" max="4" width="13.59765625" customWidth="1"/>
-    <col min="5" max="5" width="18.73046875" customWidth="1"/>
-    <col min="6" max="6" width="13.46484375" customWidth="1"/>
-    <col min="7" max="7" width="54.46484375" customWidth="1"/>
-    <col min="8" max="8" width="22.86328125" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="7" max="7" width="54.42578125" customWidth="1"/>
+    <col min="8" max="8" width="22.85546875" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="26" width="11" customWidth="1"/>
   </cols>
@@ -29401,10 +29401,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E999"/>
-  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="5" width="18.1328125" customWidth="1"/>
-    <col min="6" max="24" width="7.59765625" customWidth="1"/>
+    <col min="1" max="5" width="18.140625" customWidth="1"/>
+    <col min="6" max="24" width="7.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="12.75" customHeight="1">
@@ -30503,12 +30503,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C1000"/>
-  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11.86328125" customWidth="1"/>
-    <col min="2" max="2" width="17.59765625" customWidth="1"/>
-    <col min="3" max="3" width="30.1328125" customWidth="1"/>
-    <col min="4" max="26" width="7.59765625" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="4" max="26" width="7.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="12.75" customHeight="1">

</xml_diff>